<commit_message>
add new data for OPM, Policia and Dept. Fam
</commit_message>
<xml_diff>
--- a/data/Departamento_de_Familia/dfMalt.xlsx
+++ b/data/Departamento_de_Familia/dfMalt.xlsx
@@ -1,47 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Departamento_de_Familia\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7C98FB-6ABE-446E-818C-A71AE81C84EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10215" windowHeight="2700" activeTab="6"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2024" sheetId="7" r:id="rId1"/>
-    <sheet name="2023" sheetId="6" r:id="rId2"/>
-    <sheet name="2022" sheetId="1" r:id="rId3"/>
-    <sheet name="2021" sheetId="2" r:id="rId4"/>
-    <sheet name="2020" sheetId="3" r:id="rId5"/>
-    <sheet name="2019" sheetId="4" r:id="rId6"/>
-    <sheet name="2018" sheetId="5" r:id="rId7"/>
+    <sheet name="2025" sheetId="8" r:id="rId1"/>
+    <sheet name="2024" sheetId="7" r:id="rId2"/>
+    <sheet name="2023" sheetId="6" r:id="rId3"/>
+    <sheet name="2022" sheetId="1" r:id="rId4"/>
+    <sheet name="2021" sheetId="2" r:id="rId5"/>
+    <sheet name="2020" sheetId="3" r:id="rId6"/>
+    <sheet name="2019" sheetId="4" r:id="rId7"/>
+    <sheet name="2018" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="12">
   <si>
     <t>Tipo de Maltrato</t>
   </si>
@@ -82,7 +73,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -113,10 +104,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -396,15 +385,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E6DB18-D11D-40F3-904A-D0466F9F1C7F}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -415,122 +404,104 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>26</v>
       </c>
-      <c r="C2" s="2">
-        <v>104</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="1">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1">
-        <v>604</v>
-      </c>
-      <c r="C4" s="1">
-        <v>535</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>648</v>
+      </c>
+      <c r="C4">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
-        <v>1615</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1705</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>2154</v>
+      </c>
+      <c r="C5">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1">
-        <v>575</v>
-      </c>
-      <c r="C6" s="1">
-        <v>501</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>613</v>
+      </c>
+      <c r="C6">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>1495</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1603</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1916</v>
+      </c>
+      <c r="C7">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
-        <v>513</v>
-      </c>
-      <c r="C8" s="1">
-        <v>501</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>581</v>
+      </c>
+      <c r="C8">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="1">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1">
-        <v>21</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1">
-        <v>2</v>
-      </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -539,15 +510,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -558,122 +529,104 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2">
-        <v>75</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>26</v>
+      </c>
+      <c r="C2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1">
-        <v>531</v>
-      </c>
-      <c r="C4" s="1">
-        <v>504</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>604</v>
+      </c>
+      <c r="C4">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
-        <v>1467</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1432</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>1615</v>
+      </c>
+      <c r="C5">
+        <v>1705</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1">
-        <v>588</v>
-      </c>
-      <c r="C6" s="1">
-        <v>507</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>575</v>
+      </c>
+      <c r="C6">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>1268</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1302</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1495</v>
+      </c>
+      <c r="C7">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
-        <v>416</v>
-      </c>
-      <c r="C8" s="1">
-        <v>420</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>513</v>
+      </c>
+      <c r="C8">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="1">
-        <v>14</v>
-      </c>
-      <c r="C9" s="1">
-        <v>20</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -682,15 +635,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="3" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -701,95 +654,95 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2">
-        <v>21</v>
-      </c>
-      <c r="C2" s="2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>18</v>
+      </c>
+      <c r="C2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1">
-        <v>513</v>
-      </c>
-      <c r="C4" s="1">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>531</v>
+      </c>
+      <c r="C4">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
-        <v>1259</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1320</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>1467</v>
+      </c>
+      <c r="C5">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1">
-        <v>521</v>
-      </c>
-      <c r="C6" s="1">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>588</v>
+      </c>
+      <c r="C6">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>1156</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1272</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1268</v>
+      </c>
+      <c r="C7">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
-        <v>364</v>
-      </c>
-      <c r="C8" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>416</v>
+      </c>
+      <c r="C8">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="1">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -797,11 +750,136 @@
         <v>0</v>
       </c>
       <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="3" width="17.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>21</v>
+      </c>
+      <c r="C2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>513</v>
+      </c>
+      <c r="C4">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>1259</v>
+      </c>
+      <c r="C5">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>521</v>
+      </c>
+      <c r="C6">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1156</v>
+      </c>
+      <c r="C7">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>364</v>
+      </c>
+      <c r="C8">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:C10">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
     <sortCondition ref="A2:A10"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -809,17 +887,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -830,95 +908,95 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2">
         <v>18</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4">
         <v>483</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <v>446</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>1293</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5">
         <v>1395</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6">
         <v>633</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6">
         <v>609</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7">
         <v>1286</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7">
         <v>1380</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8">
         <v>327</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8">
         <v>299</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9">
         <v>24</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -930,135 +1008,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C10">
-    <sortCondition ref="A2:A10"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>18</v>
-      </c>
-      <c r="C2">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>539</v>
-      </c>
-      <c r="C4">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>1282</v>
-      </c>
-      <c r="C5">
-        <v>1276</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>348</v>
-      </c>
-      <c r="C6">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>1101</v>
-      </c>
-      <c r="C7">
-        <v>1123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>321</v>
-      </c>
-      <c r="C8">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9">
-        <v>19</v>
-      </c>
-      <c r="C9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState ref="A2:C10">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
     <sortCondition ref="A2:A10"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1066,16 +1016,16 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1086,95 +1036,95 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C2">
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4">
-        <v>676</v>
+        <v>539</v>
       </c>
       <c r="C4">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5">
-        <v>1628</v>
+        <v>1282</v>
       </c>
       <c r="C5">
-        <v>1543</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6">
-        <v>457</v>
+        <v>348</v>
       </c>
       <c r="C6">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7">
-        <v>1261</v>
+        <v>1101</v>
       </c>
       <c r="C7">
-        <v>1297</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>299</v>
+        <v>321</v>
       </c>
       <c r="C8">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
       <c r="B9">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1182,11 +1132,11 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C10">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
     <sortCondition ref="A2:A10"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1194,16 +1144,16 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1214,18 +1164,146 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
+        <v>26</v>
+      </c>
+      <c r="C2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>676</v>
+      </c>
+      <c r="C4">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>1628</v>
+      </c>
+      <c r="C5">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>457</v>
+      </c>
+      <c r="C6">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1261</v>
+      </c>
+      <c r="C7">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>299</v>
+      </c>
+      <c r="C8">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
+    <sortCondition ref="A2:A10"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
         <v>20</v>
       </c>
       <c r="C2">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1236,7 +1314,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1247,7 +1325,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1258,7 +1336,7 @@
         <v>1610</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1269,7 +1347,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1280,7 +1358,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1291,7 +1369,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1302,7 +1380,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1314,7 +1392,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C10">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
     <sortCondition ref="A2:A10"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>